<commit_message>
Add new Excel files for mill house mechanical equipment and extract audit. Update import script to support new file paths and enhance matching logic for equipment names and hierarchy leaves. Improve panel positioning in EquipmentMultiSelectDropdown for better UI responsiveness.
</commit_message>
<xml_diff>
--- a/docs/bi/Management-Dashboard-Formulas.xlsx
+++ b/docs/bi/Management-Dashboard-Formulas.xlsx
@@ -1,15 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E29DD855-2356-4FA5-8C75-B9D6DDAC0B4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="28665" yWindow="-135" windowWidth="29070" windowHeight="15750" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="How to read" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="1-Cell catalog" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="2-Number wise" state="visible" r:id="rId6"/>
-    <sheet sheetId="4" name="3-Filters &amp; compare" state="visible" r:id="rId7"/>
-    <sheet sheetId="5" name="4-DAX library" state="visible" r:id="rId8"/>
+    <sheet name="How to read" sheetId="1" r:id="rId1"/>
+    <sheet name="1-Cell catalog" sheetId="2" r:id="rId2"/>
+    <sheet name="2-Number wise" sheetId="3" r:id="rId3"/>
+    <sheet name="3-Filters &amp; compare" sheetId="4" r:id="rId4"/>
+    <sheet name="4-DAX library" sheetId="5" r:id="rId5"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'1-Cell catalog'!$A$1:$J$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'2-Number wise'!$A$1:$P$151</definedName>
+  </definedNames>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
@@ -1898,19 +1906,19 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="4" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="10"/>
       <color rgb="FFFFFFFF"/>
-      <sz val="10"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -2367,15 +2375,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B11"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
     <col min="2" max="2" width="110" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2383,7 +2391,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" ht="48" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
@@ -2391,7 +2399,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" ht="48" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>4</v>
       </c>
@@ -2399,7 +2407,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" ht="48" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>6</v>
       </c>
@@ -2407,7 +2415,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" ht="48" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>8</v>
       </c>
@@ -2415,7 +2423,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" ht="48" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>10</v>
       </c>
@@ -2423,7 +2431,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" ht="48" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>12</v>
       </c>
@@ -2431,7 +2439,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" ht="48" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>14</v>
       </c>
@@ -2439,7 +2447,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" ht="48" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>16</v>
       </c>
@@ -2447,7 +2455,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" ht="48" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>18</v>
       </c>
@@ -2455,7 +2463,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="11" ht="48" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>20</v>
       </c>
@@ -2465,14 +2473,15 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:J35"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="10" customWidth="1"/>
@@ -2486,7 +2495,7 @@
     <col min="10" max="10" width="40" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>22</v>
       </c>
@@ -2518,7 +2527,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="2" ht="36" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>32</v>
       </c>
@@ -2550,7 +2559,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="3" ht="36" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>32</v>
       </c>
@@ -2582,7 +2591,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="4" ht="36" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
         <v>32</v>
       </c>
@@ -2614,7 +2623,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="5" ht="36" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>32</v>
       </c>
@@ -2646,7 +2655,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="6" ht="36" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>32</v>
       </c>
@@ -2678,7 +2687,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="7" ht="36" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>32</v>
       </c>
@@ -2710,7 +2719,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="8" ht="36" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" ht="36" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
         <v>64</v>
       </c>
@@ -2742,7 +2751,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="9" ht="36" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" ht="36" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
         <v>64</v>
       </c>
@@ -2774,7 +2783,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="10" ht="36" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" ht="36" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
         <v>64</v>
       </c>
@@ -2806,7 +2815,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="11" ht="36" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" ht="36" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
         <v>64</v>
       </c>
@@ -2838,7 +2847,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="12" ht="36" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" ht="36" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
         <v>64</v>
       </c>
@@ -2870,7 +2879,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="13" ht="36" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" ht="36" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
         <v>64</v>
       </c>
@@ -2902,7 +2911,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="14" ht="36" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" ht="36" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="5" t="s">
         <v>64</v>
       </c>
@@ -2934,7 +2943,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="15" ht="36" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" ht="36" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="6" t="s">
         <v>81</v>
       </c>
@@ -2966,7 +2975,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="16" ht="36" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" ht="36" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="6" t="s">
         <v>81</v>
       </c>
@@ -2998,7 +3007,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="17" ht="36" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" ht="36" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="6" t="s">
         <v>81</v>
       </c>
@@ -3030,7 +3039,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="18" ht="36" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" ht="36" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="6" t="s">
         <v>81</v>
       </c>
@@ -3062,7 +3071,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="19" ht="36" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" ht="36" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="6" t="s">
         <v>81</v>
       </c>
@@ -3094,7 +3103,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="20" ht="36" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" ht="36" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="6" t="s">
         <v>81</v>
       </c>
@@ -3126,7 +3135,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="21" ht="36" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10" ht="36" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="6" t="s">
         <v>81</v>
       </c>
@@ -3158,7 +3167,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="22" ht="36" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:10" ht="36" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="7" t="s">
         <v>97</v>
       </c>
@@ -3190,7 +3199,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="23" ht="36" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10" ht="36" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="7" t="s">
         <v>97</v>
       </c>
@@ -3222,7 +3231,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="24" ht="36" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:10" ht="36" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="7" t="s">
         <v>97</v>
       </c>
@@ -3254,7 +3263,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="25" ht="36" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:10" ht="36" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="7" t="s">
         <v>97</v>
       </c>
@@ -3286,7 +3295,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="26" ht="36" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:10" ht="36" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="7" t="s">
         <v>97</v>
       </c>
@@ -3318,7 +3327,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="27" ht="36" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:10" ht="36" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="7" t="s">
         <v>97</v>
       </c>
@@ -3350,7 +3359,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="28" ht="36" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:10" ht="36" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="7" t="s">
         <v>97</v>
       </c>
@@ -3382,7 +3391,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="29" ht="36" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:10" ht="36" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="8" t="s">
         <v>115</v>
       </c>
@@ -3414,7 +3423,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="30" ht="36" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:10" ht="36" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="8" t="s">
         <v>115</v>
       </c>
@@ -3446,7 +3455,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="31" ht="36" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:10" ht="36" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="8" t="s">
         <v>115</v>
       </c>
@@ -3478,7 +3487,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="32" ht="36" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:10" ht="36" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="8" t="s">
         <v>115</v>
       </c>
@@ -3510,7 +3519,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="33" ht="36" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:10" ht="36" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="8" t="s">
         <v>115</v>
       </c>
@@ -3542,7 +3551,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="34" ht="36" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:10" ht="36" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="8" t="s">
         <v>115</v>
       </c>
@@ -3574,7 +3583,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="35" ht="36" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:10" ht="36" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="8" t="s">
         <v>115</v>
       </c>
@@ -3607,15 +3616,23 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:J35" xr:uid="{00000000-0001-0000-0100-000000000000}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="Cane"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:P151"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="8" customWidth="1"/>
@@ -3634,7 +3651,7 @@
     <col min="16" max="16" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>22</v>
       </c>
@@ -3684,7 +3701,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="2" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>32</v>
       </c>
@@ -3734,7 +3751,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="3" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>32</v>
       </c>
@@ -3784,7 +3801,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="4" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
         <v>32</v>
       </c>
@@ -3834,7 +3851,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="5" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>32</v>
       </c>
@@ -3884,7 +3901,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="6" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>32</v>
       </c>
@@ -3934,7 +3951,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="7" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>32</v>
       </c>
@@ -3984,7 +4001,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="8" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:16" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
         <v>32</v>
       </c>
@@ -4034,7 +4051,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="9" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:16" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
         <v>32</v>
       </c>
@@ -4084,7 +4101,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="10" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:16" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
         <v>32</v>
       </c>
@@ -4134,7 +4151,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="11" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:16" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
         <v>32</v>
       </c>
@@ -4184,7 +4201,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="12" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:16" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
         <v>32</v>
       </c>
@@ -4234,7 +4251,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="13" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:16" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
         <v>32</v>
       </c>
@@ -4284,7 +4301,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="14" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:16" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
         <v>32</v>
       </c>
@@ -4334,7 +4351,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="15" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:16" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
         <v>32</v>
       </c>
@@ -4384,7 +4401,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="16" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:16" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
         <v>32</v>
       </c>
@@ -4434,7 +4451,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="17" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
         <v>32</v>
       </c>
@@ -4484,7 +4501,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="18" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
         <v>32</v>
       </c>
@@ -4534,7 +4551,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="19" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
         <v>32</v>
       </c>
@@ -4584,7 +4601,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="20" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
         <v>32</v>
       </c>
@@ -4634,7 +4651,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="21" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
         <v>32</v>
       </c>
@@ -4684,7 +4701,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="22" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
         <v>32</v>
       </c>
@@ -4734,7 +4751,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="23" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="4" t="s">
         <v>32</v>
       </c>
@@ -4784,7 +4801,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="24" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="4" t="s">
         <v>32</v>
       </c>
@@ -4834,7 +4851,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="25" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="4" t="s">
         <v>32</v>
       </c>
@@ -4884,7 +4901,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="26" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="5" t="s">
         <v>64</v>
       </c>
@@ -4934,7 +4951,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="27" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="5" t="s">
         <v>64</v>
       </c>
@@ -4984,7 +5001,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="28" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="5" t="s">
         <v>64</v>
       </c>
@@ -5034,7 +5051,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="29" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="5" t="s">
         <v>64</v>
       </c>
@@ -5084,7 +5101,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="30" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="5" t="s">
         <v>64</v>
       </c>
@@ -5134,7 +5151,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="31" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="5" t="s">
         <v>64</v>
       </c>
@@ -5184,7 +5201,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="32" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="5" t="s">
         <v>64</v>
       </c>
@@ -5234,7 +5251,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="33" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="5" t="s">
         <v>64</v>
       </c>
@@ -5284,7 +5301,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="34" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="5" t="s">
         <v>64</v>
       </c>
@@ -5334,7 +5351,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="35" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="5" t="s">
         <v>64</v>
       </c>
@@ -5384,7 +5401,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="36" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="5" t="s">
         <v>64</v>
       </c>
@@ -5434,7 +5451,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="37" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="5" t="s">
         <v>64</v>
       </c>
@@ -5484,7 +5501,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="38" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="5" t="s">
         <v>64</v>
       </c>
@@ -5534,7 +5551,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="39" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="5" t="s">
         <v>64</v>
       </c>
@@ -5584,7 +5601,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="40" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="5" t="s">
         <v>64</v>
       </c>
@@ -5634,7 +5651,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="41" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="5" t="s">
         <v>64</v>
       </c>
@@ -5684,7 +5701,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="42" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="5" t="s">
         <v>64</v>
       </c>
@@ -5734,7 +5751,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="43" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="5" t="s">
         <v>64</v>
       </c>
@@ -5784,7 +5801,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="44" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="5" t="s">
         <v>64</v>
       </c>
@@ -5834,7 +5851,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="45" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="5" t="s">
         <v>64</v>
       </c>
@@ -5884,7 +5901,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="46" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="5" t="s">
         <v>64</v>
       </c>
@@ -5934,7 +5951,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="47" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="5" t="s">
         <v>64</v>
       </c>
@@ -5984,7 +6001,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="48" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="5" t="s">
         <v>64</v>
       </c>
@@ -6034,7 +6051,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="49" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="5" t="s">
         <v>64</v>
       </c>
@@ -6084,7 +6101,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="50" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="5" t="s">
         <v>64</v>
       </c>
@@ -6134,7 +6151,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="51" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="5" t="s">
         <v>64</v>
       </c>
@@ -6184,7 +6201,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="52" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="5" t="s">
         <v>64</v>
       </c>
@@ -6234,7 +6251,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="53" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="6" t="s">
         <v>81</v>
       </c>
@@ -6284,7 +6301,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="54" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="6" t="s">
         <v>81</v>
       </c>
@@ -6334,7 +6351,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="55" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" s="6" t="s">
         <v>81</v>
       </c>
@@ -6384,7 +6401,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="56" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A56" s="6" t="s">
         <v>81</v>
       </c>
@@ -6434,7 +6451,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="57" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A57" s="6" t="s">
         <v>81</v>
       </c>
@@ -6484,7 +6501,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="58" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A58" s="6" t="s">
         <v>81</v>
       </c>
@@ -6534,7 +6551,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="59" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A59" s="6" t="s">
         <v>81</v>
       </c>
@@ -6584,7 +6601,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="60" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A60" s="6" t="s">
         <v>81</v>
       </c>
@@ -6634,7 +6651,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="61" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A61" s="6" t="s">
         <v>81</v>
       </c>
@@ -6684,7 +6701,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="62" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A62" s="6" t="s">
         <v>81</v>
       </c>
@@ -6734,7 +6751,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="63" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A63" s="6" t="s">
         <v>81</v>
       </c>
@@ -6784,7 +6801,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="64" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A64" s="6" t="s">
         <v>81</v>
       </c>
@@ -6834,7 +6851,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="65" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A65" s="6" t="s">
         <v>81</v>
       </c>
@@ -6884,7 +6901,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="66" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A66" s="6" t="s">
         <v>81</v>
       </c>
@@ -6934,7 +6951,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="67" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A67" s="6" t="s">
         <v>81</v>
       </c>
@@ -6984,7 +7001,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="68" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A68" s="6" t="s">
         <v>81</v>
       </c>
@@ -7034,7 +7051,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="69" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A69" s="6" t="s">
         <v>81</v>
       </c>
@@ -7084,7 +7101,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="70" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A70" s="6" t="s">
         <v>81</v>
       </c>
@@ -7134,7 +7151,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="71" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A71" s="6" t="s">
         <v>81</v>
       </c>
@@ -7184,7 +7201,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="72" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A72" s="6" t="s">
         <v>81</v>
       </c>
@@ -7234,7 +7251,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="73" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A73" s="6" t="s">
         <v>81</v>
       </c>
@@ -7284,7 +7301,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="74" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A74" s="6" t="s">
         <v>81</v>
       </c>
@@ -7334,7 +7351,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="75" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A75" s="6" t="s">
         <v>81</v>
       </c>
@@ -7384,7 +7401,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="76" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A76" s="6" t="s">
         <v>81</v>
       </c>
@@ -7434,7 +7451,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="77" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A77" s="6" t="s">
         <v>81</v>
       </c>
@@ -7484,7 +7501,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="78" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A78" s="6" t="s">
         <v>81</v>
       </c>
@@ -7534,7 +7551,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="79" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A79" s="6" t="s">
         <v>81</v>
       </c>
@@ -7584,7 +7601,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="80" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A80" s="6" t="s">
         <v>81</v>
       </c>
@@ -7634,7 +7651,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="81" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A81" s="6" t="s">
         <v>81</v>
       </c>
@@ -7684,7 +7701,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="82" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A82" s="6" t="s">
         <v>81</v>
       </c>
@@ -7734,7 +7751,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="83" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A83" s="6" t="s">
         <v>81</v>
       </c>
@@ -7784,7 +7801,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="84" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A84" s="6" t="s">
         <v>81</v>
       </c>
@@ -7834,7 +7851,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="85" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A85" s="6" t="s">
         <v>81</v>
       </c>
@@ -7884,7 +7901,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="86" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A86" s="6" t="s">
         <v>81</v>
       </c>
@@ -7934,7 +7951,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="87" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A87" s="6" t="s">
         <v>81</v>
       </c>
@@ -7984,7 +8001,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="88" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A88" s="6" t="s">
         <v>81</v>
       </c>
@@ -8034,7 +8051,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="89" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A89" s="7" t="s">
         <v>97</v>
       </c>
@@ -8084,7 +8101,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="90" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A90" s="7" t="s">
         <v>97</v>
       </c>
@@ -8134,7 +8151,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="91" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A91" s="7" t="s">
         <v>97</v>
       </c>
@@ -8184,7 +8201,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="92" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A92" s="7" t="s">
         <v>97</v>
       </c>
@@ -8234,7 +8251,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="93" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A93" s="7" t="s">
         <v>97</v>
       </c>
@@ -8284,7 +8301,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="94" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A94" s="7" t="s">
         <v>97</v>
       </c>
@@ -8334,7 +8351,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="95" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A95" s="7" t="s">
         <v>97</v>
       </c>
@@ -8384,7 +8401,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="96" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A96" s="7" t="s">
         <v>97</v>
       </c>
@@ -8434,7 +8451,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="97" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A97" s="7" t="s">
         <v>97</v>
       </c>
@@ -8484,7 +8501,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="98" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A98" s="7" t="s">
         <v>97</v>
       </c>
@@ -8534,7 +8551,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="99" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A99" s="7" t="s">
         <v>97</v>
       </c>
@@ -8584,7 +8601,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="100" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A100" s="7" t="s">
         <v>97</v>
       </c>
@@ -8634,7 +8651,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="101" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A101" s="7" t="s">
         <v>97</v>
       </c>
@@ -8684,7 +8701,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="102" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A102" s="7" t="s">
         <v>97</v>
       </c>
@@ -8734,7 +8751,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="103" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A103" s="7" t="s">
         <v>97</v>
       </c>
@@ -8784,7 +8801,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="104" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A104" s="7" t="s">
         <v>97</v>
       </c>
@@ -8834,7 +8851,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="105" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A105" s="7" t="s">
         <v>97</v>
       </c>
@@ -8884,7 +8901,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="106" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A106" s="7" t="s">
         <v>97</v>
       </c>
@@ -8934,7 +8951,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="107" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A107" s="7" t="s">
         <v>97</v>
       </c>
@@ -8984,7 +9001,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="108" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A108" s="7" t="s">
         <v>97</v>
       </c>
@@ -9034,7 +9051,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="109" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A109" s="7" t="s">
         <v>97</v>
       </c>
@@ -9084,7 +9101,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="110" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A110" s="7" t="s">
         <v>97</v>
       </c>
@@ -9134,7 +9151,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="111" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A111" s="7" t="s">
         <v>97</v>
       </c>
@@ -9184,7 +9201,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="112" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A112" s="7" t="s">
         <v>97</v>
       </c>
@@ -9234,7 +9251,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="113" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A113" s="7" t="s">
         <v>97</v>
       </c>
@@ -9284,7 +9301,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="114" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A114" s="7" t="s">
         <v>97</v>
       </c>
@@ -9334,7 +9351,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="115" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A115" s="7" t="s">
         <v>97</v>
       </c>
@@ -9384,7 +9401,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="116" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A116" s="7" t="s">
         <v>97</v>
       </c>
@@ -9434,7 +9451,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="117" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A117" s="7" t="s">
         <v>97</v>
       </c>
@@ -9484,7 +9501,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="118" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A118" s="7" t="s">
         <v>97</v>
       </c>
@@ -9534,7 +9551,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="119" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A119" s="7" t="s">
         <v>97</v>
       </c>
@@ -9584,7 +9601,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="120" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A120" s="7" t="s">
         <v>97</v>
       </c>
@@ -9634,7 +9651,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="121" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A121" s="7" t="s">
         <v>97</v>
       </c>
@@ -9684,7 +9701,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="122" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A122" s="8" t="s">
         <v>115</v>
       </c>
@@ -9734,7 +9751,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="123" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A123" s="8" t="s">
         <v>115</v>
       </c>
@@ -9784,7 +9801,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="124" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A124" s="8" t="s">
         <v>115</v>
       </c>
@@ -9834,7 +9851,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="125" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A125" s="8" t="s">
         <v>115</v>
       </c>
@@ -9884,7 +9901,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="126" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A126" s="8" t="s">
         <v>115</v>
       </c>
@@ -9934,7 +9951,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="127" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A127" s="8" t="s">
         <v>115</v>
       </c>
@@ -9984,7 +10001,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="128" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A128" s="8" t="s">
         <v>115</v>
       </c>
@@ -10034,7 +10051,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="129" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A129" s="8" t="s">
         <v>115</v>
       </c>
@@ -10084,7 +10101,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="130" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A130" s="8" t="s">
         <v>115</v>
       </c>
@@ -10134,7 +10151,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="131" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A131" s="8" t="s">
         <v>115</v>
       </c>
@@ -10184,7 +10201,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="132" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A132" s="8" t="s">
         <v>115</v>
       </c>
@@ -10234,7 +10251,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="133" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A133" s="8" t="s">
         <v>115</v>
       </c>
@@ -10284,7 +10301,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="134" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A134" s="8" t="s">
         <v>115</v>
       </c>
@@ -10334,7 +10351,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="135" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A135" s="8" t="s">
         <v>115</v>
       </c>
@@ -10384,7 +10401,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="136" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A136" s="8" t="s">
         <v>115</v>
       </c>
@@ -10434,7 +10451,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="137" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A137" s="8" t="s">
         <v>115</v>
       </c>
@@ -10484,7 +10501,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="138" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A138" s="8" t="s">
         <v>115</v>
       </c>
@@ -10534,7 +10551,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="139" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A139" s="8" t="s">
         <v>115</v>
       </c>
@@ -10584,7 +10601,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="140" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A140" s="8" t="s">
         <v>115</v>
       </c>
@@ -10634,7 +10651,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="141" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A141" s="8" t="s">
         <v>115</v>
       </c>
@@ -10684,7 +10701,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="142" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A142" s="8" t="s">
         <v>115</v>
       </c>
@@ -10734,7 +10751,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="143" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A143" s="8" t="s">
         <v>115</v>
       </c>
@@ -10784,7 +10801,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="144" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A144" s="8" t="s">
         <v>115</v>
       </c>
@@ -10834,7 +10851,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="145" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A145" s="8" t="s">
         <v>115</v>
       </c>
@@ -10884,7 +10901,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="146" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A146" s="8" t="s">
         <v>115</v>
       </c>
@@ -10934,7 +10951,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="147" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A147" s="8" t="s">
         <v>115</v>
       </c>
@@ -10984,7 +11001,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="148" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A148" s="8" t="s">
         <v>115</v>
       </c>
@@ -11034,7 +11051,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="149" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A149" s="8" t="s">
         <v>115</v>
       </c>
@@ -11084,7 +11101,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="150" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A150" s="8" t="s">
         <v>115</v>
       </c>
@@ -11134,7 +11151,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="151" ht="42" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:16" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A151" s="8" t="s">
         <v>115</v>
       </c>
@@ -11185,15 +11202,27 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:P151" xr:uid="{00000000-0001-0000-0200-000000000000}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="Cane"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="2">
+      <filters>
+        <filter val="Yard Bal. (8AM)"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:E9"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
     <col min="2" max="2" width="42" customWidth="1"/>
@@ -11202,7 +11231,7 @@
     <col min="5" max="5" width="70" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>547</v>
       </c>
@@ -11219,7 +11248,7 @@
         <v>551</v>
       </c>
     </row>
-    <row r="2" ht="36" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>552</v>
       </c>
@@ -11236,7 +11265,7 @@
         <v>556</v>
       </c>
     </row>
-    <row r="3" ht="36" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>557</v>
       </c>
@@ -11253,7 +11282,7 @@
         <v>561</v>
       </c>
     </row>
-    <row r="4" ht="36" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>562</v>
       </c>
@@ -11270,7 +11299,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="5" ht="36" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>566</v>
       </c>
@@ -11287,7 +11316,7 @@
         <v>570</v>
       </c>
     </row>
-    <row r="6" ht="36" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>571</v>
       </c>
@@ -11304,7 +11333,7 @@
         <v>575</v>
       </c>
     </row>
-    <row r="7" ht="36" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>576</v>
       </c>
@@ -11321,7 +11350,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="8" ht="36" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>581</v>
       </c>
@@ -11338,7 +11367,7 @@
         <v>584</v>
       </c>
     </row>
-    <row r="9" ht="36" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>585</v>
       </c>
@@ -11357,21 +11386,21 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
     <col min="2" max="2" width="95" customWidth="1"/>
     <col min="3" max="3" width="50" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>587</v>
       </c>
@@ -11382,7 +11411,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="2" ht="36" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>590</v>
       </c>
@@ -11393,7 +11422,7 @@
         <v>592</v>
       </c>
     </row>
-    <row r="3" ht="36" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>593</v>
       </c>
@@ -11404,7 +11433,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="4" ht="36" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>596</v>
       </c>
@@ -11415,7 +11444,7 @@
         <v>598</v>
       </c>
     </row>
-    <row r="5" ht="36" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>599</v>
       </c>
@@ -11426,7 +11455,7 @@
         <v>601</v>
       </c>
     </row>
-    <row r="6" ht="36" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>602</v>
       </c>
@@ -11437,7 +11466,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="7" ht="36" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>605</v>
       </c>
@@ -11448,7 +11477,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="8" ht="36" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>608</v>
       </c>
@@ -11459,7 +11488,7 @@
         <v>610</v>
       </c>
     </row>
-    <row r="9" ht="36" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>611</v>
       </c>
@@ -11470,7 +11499,7 @@
         <v>613</v>
       </c>
     </row>
-    <row r="10" ht="36" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>614</v>
       </c>
@@ -11481,7 +11510,7 @@
         <v>616</v>
       </c>
     </row>
-    <row r="11" ht="36" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>617</v>
       </c>
@@ -11492,7 +11521,7 @@
         <v>619</v>
       </c>
     </row>
-    <row r="12" ht="36" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>620</v>
       </c>
@@ -11503,7 +11532,7 @@
         <v>622</v>
       </c>
     </row>
-    <row r="13" ht="36" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" ht="36" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>623</v>
       </c>
@@ -11516,6 +11545,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>